<commit_message>
remove and reupload code for Chrome Extensions and Python projects
</commit_message>
<xml_diff>
--- a/气象/分站资料/俄罗斯/外贝加尔边疆区冷站阈值天数.xlsx
+++ b/气象/分站资料/俄罗斯/外贝加尔边疆区冷站阈值天数.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\文档\GIT SYNC\default\气象\分站资料\俄罗斯\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912ADE82-1A72-46DC-B30C-33DB409020F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A00E711F-24E6-41EA-AE0E-448EC4AB905B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D308DEC9-CED1-4015-BAB2-E937FD661EDE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{D308DEC9-CED1-4015-BAB2-E937FD661EDE}"/>
   </bookViews>
   <sheets>
     <sheet name="中卡拉尔" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="192">
   <si>
     <t>冬季</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -43,208 +43,6 @@
   <si>
     <t>零下50度天数</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>共 66 冬</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1959~1960冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1960~1961冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1961~1962冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1962~1963冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1963~1964冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1964~1965冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1965~1966冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1966~1967冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1967~1968冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1968~1969冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1969~1970冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1970~1971冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1971~1972冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1972~1973冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1973~1974冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1974~1975冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1975~1976冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1976~1977冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1977~1978冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1978~1979冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1979~1980冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1980~1981冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1981~1982冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1982~1983冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1983~1984冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1984~1985冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1985~1986冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1986~1987冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1987~1988冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1988~1989冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1989~1990冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1990~1991冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1991~1992冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1992~1993冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1993~1994冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1994~1995冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1995~1996冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1996~1997冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1997~1998冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1998~1999冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 1999~2000冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2000~2001冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2001~2002冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2002~2003冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2003~2004冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2004~2005冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2005~2006冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2006~2007冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2007~2008冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2008~2009冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2009~2010冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2010~2011冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2011~2012冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2012~2013冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2013~2014冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2014~2015冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2015~2016冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2016~2017冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2017~2018冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2018~2019冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2019~2020冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2020~2021冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2021~2022冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2022~2023冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2023~2024冬</t>
-  </si>
-  <si>
-    <t>乌斯季卡连加 2024~2025冬</t>
   </si>
   <si>
     <t>共 17 天低温达到 -50℃</t>
@@ -351,94 +149,6 @@
   </si>
   <si>
     <t>无 -50℃</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="32"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>乌斯季卡连加</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="32"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>各冬低温(零下50度版)</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="24"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>乌斯季卡连加</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:    东经116.517°,  北纬54.45°,  海拔686m.  俄罗斯</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>外贝加尔边疆区</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>通戈科琴斯基区</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>最低</t>
@@ -930,6 +640,307 @@
       </rPr>
       <t>卡拉斯基区</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>无 -50℃</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1959~1960冬</t>
+  </si>
+  <si>
+    <t>1960~1961冬</t>
+  </si>
+  <si>
+    <t>1961~1962冬</t>
+  </si>
+  <si>
+    <t>1962~1963冬</t>
+  </si>
+  <si>
+    <t>1963~1964冬</t>
+  </si>
+  <si>
+    <t>1964~1965冬</t>
+  </si>
+  <si>
+    <t>1965~1966冬</t>
+  </si>
+  <si>
+    <t>1966~1967冬</t>
+  </si>
+  <si>
+    <t>1967~1968冬</t>
+  </si>
+  <si>
+    <t>1968~1969冬</t>
+  </si>
+  <si>
+    <t>1969~1970冬</t>
+  </si>
+  <si>
+    <t>1970~1971冬</t>
+  </si>
+  <si>
+    <t>1971~1972冬</t>
+  </si>
+  <si>
+    <t>1972~1973冬</t>
+  </si>
+  <si>
+    <t>1973~1974冬</t>
+  </si>
+  <si>
+    <t>1974~1975冬</t>
+  </si>
+  <si>
+    <t>1975~1976冬</t>
+  </si>
+  <si>
+    <t>1976~1977冬</t>
+  </si>
+  <si>
+    <t>1977~1978冬</t>
+  </si>
+  <si>
+    <t>1978~1979冬</t>
+  </si>
+  <si>
+    <t>1979~1980冬</t>
+  </si>
+  <si>
+    <t>1980~1981冬</t>
+  </si>
+  <si>
+    <t>1981~1982冬</t>
+  </si>
+  <si>
+    <t>1982~1983冬</t>
+  </si>
+  <si>
+    <t>1983~1984冬</t>
+  </si>
+  <si>
+    <t>1984~1985冬</t>
+  </si>
+  <si>
+    <t>1985~1986冬</t>
+  </si>
+  <si>
+    <t>1986~1987冬</t>
+  </si>
+  <si>
+    <t>1987~1988冬</t>
+  </si>
+  <si>
+    <t>1988~1989冬</t>
+  </si>
+  <si>
+    <t>1989~1990冬</t>
+  </si>
+  <si>
+    <t>1990~1991冬</t>
+  </si>
+  <si>
+    <t>1991~1992冬</t>
+  </si>
+  <si>
+    <t>1992~1993冬</t>
+  </si>
+  <si>
+    <t>1993~1994冬</t>
+  </si>
+  <si>
+    <t>1994~1995冬</t>
+  </si>
+  <si>
+    <t>1995~1996冬</t>
+  </si>
+  <si>
+    <t>1996~1997冬</t>
+  </si>
+  <si>
+    <t>1997~1998冬</t>
+  </si>
+  <si>
+    <t>1998~1999冬</t>
+  </si>
+  <si>
+    <t>1999~2000冬</t>
+  </si>
+  <si>
+    <t>2000~2001冬</t>
+  </si>
+  <si>
+    <t>2001~2002冬</t>
+  </si>
+  <si>
+    <t>2002~2003冬</t>
+  </si>
+  <si>
+    <t>2003~2004冬</t>
+  </si>
+  <si>
+    <t>2004~2005冬</t>
+  </si>
+  <si>
+    <t>2005~2006冬</t>
+  </si>
+  <si>
+    <t>2006~2007冬</t>
+  </si>
+  <si>
+    <t>2007~2008冬</t>
+  </si>
+  <si>
+    <t>2008~2009冬</t>
+  </si>
+  <si>
+    <t>2009~2010冬</t>
+  </si>
+  <si>
+    <t>2010~2011冬</t>
+  </si>
+  <si>
+    <t>2011~2012冬</t>
+  </si>
+  <si>
+    <t>2012~2013冬</t>
+  </si>
+  <si>
+    <t>2013~2014冬</t>
+  </si>
+  <si>
+    <t>2014~2015冬</t>
+  </si>
+  <si>
+    <t>2015~2016冬</t>
+  </si>
+  <si>
+    <t>2016~2017冬</t>
+  </si>
+  <si>
+    <t>2017~2018冬</t>
+  </si>
+  <si>
+    <t>2018~2019冬</t>
+  </si>
+  <si>
+    <t>2019~2020冬</t>
+  </si>
+  <si>
+    <t>2020~2021冬</t>
+  </si>
+  <si>
+    <t>2021~2022冬</t>
+  </si>
+  <si>
+    <t>2022~2023冬</t>
+  </si>
+  <si>
+    <t>2023~2024冬</t>
+  </si>
+  <si>
+    <t>2024~2025冬</t>
+  </si>
+  <si>
+    <t>2025~2026冬</t>
+  </si>
+  <si>
+    <t>共 67 冬</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="32"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>乌斯季卡连加</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="32"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-50℃气温天数</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>乌斯季卡连加</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:    54.45°N,  116.517°E,  686m,  俄罗斯</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>外贝加尔边疆区</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>通戈科琴斯基区,  人口143(2021)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>低温-50℃天数</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1270,7 +1281,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1385,15 +1396,27 @@
     <xf numFmtId="176" fontId="9" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1415,25 +1438,16 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="12" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1779,52 +1793,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
-        <v>188</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
+      <c r="A1" s="48" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
     </row>
     <row r="2" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="41"/>
       <c r="D2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="46" t="s">
-        <v>187</v>
-      </c>
-      <c r="I2" s="47"/>
+      <c r="E2" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="44"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2" s="51"/>
     </row>
     <row r="3" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E3" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F3" s="33">
         <v>-49.7</v>
@@ -1833,28 +1847,28 @@
         <v>14252</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I3" s="29" t="s">
-        <v>180</v>
+        <v>112</v>
       </c>
       <c r="O3" s="26"/>
     </row>
     <row r="4" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F4" s="33">
         <v>-49.2</v>
@@ -1863,28 +1877,28 @@
         <v>14614</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I4" s="29" t="s">
-        <v>181</v>
+        <v>113</v>
       </c>
       <c r="O4" s="26"/>
     </row>
     <row r="5" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>164</v>
+        <v>96</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F5" s="33">
         <v>-55.9</v>
@@ -1898,19 +1912,19 @@
     </row>
     <row r="6" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F6" s="33">
         <v>-51.1</v>
@@ -1919,57 +1933,57 @@
         <v>15307</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>182</v>
+        <v>114</v>
       </c>
       <c r="O6" s="26"/>
     </row>
     <row r="7" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F7" s="33">
         <v>-49.7</v>
       </c>
       <c r="G7" s="36" t="s">
-        <v>175</v>
+        <v>107</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I7" s="29" t="s">
-        <v>184</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E8" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F8" s="33">
         <v>-48.7</v>
@@ -1978,28 +1992,28 @@
         <v>16064</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>185</v>
+        <v>117</v>
       </c>
       <c r="O8" s="26"/>
     </row>
     <row r="9" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F9" s="33">
         <v>-50.2</v>
@@ -2008,28 +2022,28 @@
         <v>16461</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>186</v>
+        <v>118</v>
       </c>
       <c r="O9" s="26"/>
     </row>
     <row r="10" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F10" s="33">
         <v>-51.6</v>
@@ -2043,19 +2057,19 @@
     </row>
     <row r="11" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>165</v>
+        <v>97</v>
       </c>
       <c r="E11" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F11" s="33">
         <v>-53.1</v>
@@ -2069,19 +2083,19 @@
     </row>
     <row r="12" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F12" s="33">
         <v>-50.2</v>
@@ -2095,19 +2109,19 @@
     </row>
     <row r="13" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F13" s="33">
         <v>-51.1</v>
@@ -2121,19 +2135,19 @@
     </row>
     <row r="14" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F14" s="33">
         <v>-51</v>
@@ -2147,19 +2161,19 @@
     </row>
     <row r="15" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>165</v>
+        <v>97</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F15" s="33">
         <v>-54.7</v>
@@ -2173,19 +2187,19 @@
     </row>
     <row r="16" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="E16" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F16" s="33">
         <v>-52</v>
@@ -2199,19 +2213,19 @@
     </row>
     <row r="17" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>166</v>
+        <v>98</v>
       </c>
       <c r="E17" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F17" s="37">
         <v>-56.2</v>
@@ -2225,19 +2239,19 @@
     </row>
     <row r="18" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>101</v>
+        <v>33</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>167</v>
+        <v>99</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F18" s="33">
         <v>-51.6</v>
@@ -2251,19 +2265,19 @@
     </row>
     <row r="19" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>102</v>
+        <v>34</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E19" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F19" s="33">
         <v>-50.2</v>
@@ -2277,19 +2291,19 @@
     </row>
     <row r="20" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>167</v>
+        <v>99</v>
       </c>
       <c r="E20" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F20" s="33">
         <v>-51.8</v>
@@ -2303,19 +2317,19 @@
     </row>
     <row r="21" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>104</v>
+        <v>36</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E21" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F21" s="33">
         <v>-49.8</v>
@@ -2329,19 +2343,19 @@
     </row>
     <row r="22" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>105</v>
+        <v>37</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>168</v>
+        <v>100</v>
       </c>
       <c r="E22" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F22" s="33">
         <v>-52.1</v>
@@ -2355,19 +2369,19 @@
     </row>
     <row r="23" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="E23" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F23" s="33">
         <v>-55.2</v>
@@ -2381,19 +2395,19 @@
     </row>
     <row r="24" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>169</v>
+        <v>101</v>
       </c>
       <c r="E24" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F24" s="33">
         <v>-54.1</v>
@@ -2407,19 +2421,19 @@
     </row>
     <row r="25" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F25" s="33">
         <v>-52.2</v>
@@ -2433,19 +2447,19 @@
     </row>
     <row r="26" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>109</v>
+        <v>41</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F26" s="33">
         <v>-51.1</v>
@@ -2459,19 +2473,19 @@
     </row>
     <row r="27" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>110</v>
+        <v>42</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E27" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F27" s="33">
         <v>-48.8</v>
@@ -2485,19 +2499,19 @@
     </row>
     <row r="28" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E28" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F28" s="33">
         <v>-47.8</v>
@@ -2511,19 +2525,19 @@
     </row>
     <row r="29" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>112</v>
+        <v>44</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E29" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F29" s="33">
         <v>-51.2</v>
@@ -2537,19 +2551,19 @@
     </row>
     <row r="30" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>113</v>
+        <v>45</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>170</v>
+        <v>102</v>
       </c>
       <c r="E30" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F30" s="33">
         <v>-55.8</v>
@@ -2563,19 +2577,19 @@
     </row>
     <row r="31" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>114</v>
+        <v>46</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E31" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F31" s="33">
         <v>-48.8</v>
@@ -2589,19 +2603,19 @@
     </row>
     <row r="32" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>115</v>
+        <v>47</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E32" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F32" s="33">
         <v>-48.9</v>
@@ -2615,19 +2629,19 @@
     </row>
     <row r="33" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>171</v>
+        <v>103</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F33" s="33">
         <v>-55.7</v>
@@ -2641,19 +2655,19 @@
     </row>
     <row r="34" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>117</v>
+        <v>49</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E34" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F34" s="33">
         <v>-48.4</v>
@@ -2667,44 +2681,44 @@
     </row>
     <row r="35" spans="1:15" ht="52.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="E35" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F35" s="33">
         <v>-51.5</v>
       </c>
       <c r="G35" s="36" t="s">
-        <v>176</v>
+        <v>108</v>
       </c>
       <c r="H35" s="31"/>
       <c r="I35" s="29"/>
     </row>
     <row r="36" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>119</v>
+        <v>51</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E36" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F36" s="33">
         <v>-48.7</v>
@@ -2718,19 +2732,19 @@
     </row>
     <row r="37" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>120</v>
+        <v>52</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E37" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F37" s="33">
         <v>-53</v>
@@ -2744,19 +2758,19 @@
     </row>
     <row r="38" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>121</v>
+        <v>53</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="E38" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F38" s="33">
         <v>-52.1</v>
@@ -2770,19 +2784,19 @@
     </row>
     <row r="39" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>122</v>
+        <v>54</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="E39" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F39" s="33">
         <v>-50.9</v>
@@ -2796,19 +2810,19 @@
     </row>
     <row r="40" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>123</v>
+        <v>55</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E40" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F40" s="33">
         <v>-50</v>
@@ -2822,19 +2836,19 @@
     </row>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="E41" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F41" s="33">
         <v>-52.1</v>
@@ -2848,19 +2862,19 @@
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>125</v>
+        <v>57</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E42" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F42" s="33">
         <v>-50.2</v>
@@ -2874,19 +2888,19 @@
     </row>
     <row r="43" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="E43" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F43" s="33">
         <v>-54.3</v>
@@ -2900,19 +2914,19 @@
     </row>
     <row r="44" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>127</v>
+        <v>59</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E44" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F44" s="33">
         <v>-53.9</v>
@@ -2926,19 +2940,19 @@
     </row>
     <row r="45" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>128</v>
+        <v>60</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E45" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F45" s="33">
         <v>-48.3</v>
@@ -2952,19 +2966,19 @@
     </row>
     <row r="46" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>129</v>
+        <v>61</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E46" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F46" s="33">
         <v>-49.9</v>
@@ -2978,19 +2992,19 @@
     </row>
     <row r="47" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>130</v>
+        <v>62</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E47" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F47" s="33">
         <v>-48.1</v>
@@ -3004,19 +3018,19 @@
     </row>
     <row r="48" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>131</v>
+        <v>63</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E48" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F48" s="33">
         <v>-47.8</v>
@@ -3030,19 +3044,19 @@
     </row>
     <row r="49" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E49" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F49" s="33">
         <v>-52.2</v>
@@ -3056,19 +3070,19 @@
     </row>
     <row r="50" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>133</v>
+        <v>65</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E50" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F50" s="33">
         <v>-48.5</v>
@@ -3082,19 +3096,19 @@
     </row>
     <row r="51" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>134</v>
+        <v>66</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>169</v>
+        <v>101</v>
       </c>
       <c r="E51" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F51" s="33">
         <v>-55</v>
@@ -3108,19 +3122,19 @@
     </row>
     <row r="52" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B52" s="23" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E52" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F52" s="33">
         <v>-51.6</v>
@@ -3134,19 +3148,19 @@
     </row>
     <row r="53" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A53" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B53" s="23" t="s">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E53" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F53" s="37">
         <v>-45.6</v>
@@ -3160,44 +3174,44 @@
     </row>
     <row r="54" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>137</v>
+        <v>69</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E54" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F54" s="33">
         <v>-49.7</v>
       </c>
       <c r="G54" s="36" t="s">
-        <v>177</v>
+        <v>109</v>
       </c>
       <c r="H54" s="31"/>
       <c r="I54" s="29"/>
     </row>
     <row r="55" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A55" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E55" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F55" s="33">
         <v>-47.2</v>
@@ -3211,19 +3225,19 @@
     </row>
     <row r="56" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A56" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>139</v>
+        <v>71</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E56" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F56" s="33">
         <v>-47.4</v>
@@ -3237,19 +3251,19 @@
     </row>
     <row r="57" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A57" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B57" s="23" t="s">
-        <v>140</v>
+        <v>72</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E57" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F57" s="33">
         <v>-45.7</v>
@@ -3263,19 +3277,19 @@
     </row>
     <row r="58" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A58" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B58" s="23" t="s">
-        <v>141</v>
+        <v>73</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E58" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F58" s="33">
         <v>-51.2</v>
@@ -3289,19 +3303,19 @@
     </row>
     <row r="59" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A59" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B59" s="23" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E59" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F59" s="33">
         <v>-45.8</v>
@@ -3315,19 +3329,19 @@
     </row>
     <row r="60" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A60" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B60" s="23" t="s">
-        <v>143</v>
+        <v>75</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E60" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F60" s="33">
         <v>-50.2</v>
@@ -3341,19 +3355,19 @@
     </row>
     <row r="61" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A61" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B61" s="23" t="s">
-        <v>144</v>
+        <v>76</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>164</v>
+        <v>96</v>
       </c>
       <c r="E61" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F61" s="33">
         <v>-54.6</v>
@@ -3367,19 +3381,19 @@
     </row>
     <row r="62" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A62" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B62" s="23" t="s">
-        <v>145</v>
+        <v>77</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="E62" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F62" s="33">
         <v>-51.3</v>
@@ -3393,19 +3407,19 @@
     </row>
     <row r="63" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A63" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B63" s="23" t="s">
-        <v>146</v>
+        <v>78</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E63" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F63" s="33">
         <v>-49.4</v>
@@ -3419,44 +3433,44 @@
     </row>
     <row r="64" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A64" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B64" s="23" t="s">
-        <v>147</v>
+        <v>79</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E64" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F64" s="33">
         <v>-47.9</v>
       </c>
       <c r="G64" s="36" t="s">
-        <v>178</v>
+        <v>110</v>
       </c>
       <c r="H64" s="31"/>
       <c r="I64" s="29"/>
     </row>
     <row r="65" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A65" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B65" s="23" t="s">
-        <v>148</v>
+        <v>80</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="E65" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F65" s="33">
         <v>-50.8</v>
@@ -3470,19 +3484,19 @@
     </row>
     <row r="66" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A66" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B66" s="23" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="C66" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E66" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F66" s="33">
         <v>-46.5</v>
@@ -3496,19 +3510,19 @@
     </row>
     <row r="67" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A67" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B67" s="23" t="s">
-        <v>150</v>
+        <v>82</v>
       </c>
       <c r="C67" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E67" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F67" s="33">
         <v>-50.8</v>
@@ -3522,19 +3536,19 @@
     </row>
     <row r="68" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A68" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B68" s="23" t="s">
-        <v>151</v>
+        <v>83</v>
       </c>
       <c r="C68" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E68" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F68" s="33">
         <v>-45.9</v>
@@ -3548,19 +3562,19 @@
     </row>
     <row r="69" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A69" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B69" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="B69" s="23" t="s">
-        <v>152</v>
-      </c>
       <c r="C69" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E69" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F69" s="33">
         <v>-46.3</v>
@@ -3574,19 +3588,19 @@
     </row>
     <row r="70" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A70" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B70" s="23" t="s">
-        <v>153</v>
+        <v>85</v>
       </c>
       <c r="C70" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="E70" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F70" s="33">
         <v>-50.5</v>
@@ -3600,19 +3614,19 @@
     </row>
     <row r="71" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A71" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B71" s="23" t="s">
-        <v>154</v>
+        <v>86</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E71" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F71" s="33">
         <v>-49.3</v>
@@ -3626,19 +3640,19 @@
     </row>
     <row r="72" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A72" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B72" s="23" t="s">
-        <v>155</v>
+        <v>87</v>
       </c>
       <c r="C72" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E72" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F72" s="33">
         <v>-49.7</v>
@@ -3652,19 +3666,19 @@
     </row>
     <row r="73" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A73" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B73" s="23" t="s">
-        <v>156</v>
+        <v>88</v>
       </c>
       <c r="C73" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E73" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F73" s="33">
         <v>-48</v>
@@ -3678,19 +3692,19 @@
     </row>
     <row r="74" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A74" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B74" s="23" t="s">
-        <v>157</v>
+        <v>89</v>
       </c>
       <c r="C74" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D74" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E74" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F74" s="33">
         <v>-46.8</v>
@@ -3704,19 +3718,19 @@
     </row>
     <row r="75" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A75" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B75" s="23" t="s">
-        <v>158</v>
+        <v>90</v>
       </c>
       <c r="C75" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E75" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F75" s="33">
         <v>-49.3</v>
@@ -3730,19 +3744,19 @@
     </row>
     <row r="76" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A76" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>159</v>
+        <v>91</v>
       </c>
       <c r="C76" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E76" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F76" s="33">
         <v>-49.1</v>
@@ -3756,44 +3770,44 @@
     </row>
     <row r="77" spans="1:15" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A77" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B77" s="23" t="s">
-        <v>160</v>
+        <v>92</v>
       </c>
       <c r="C77" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E77" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F77" s="33">
         <v>-48.9</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>179</v>
+        <v>111</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="29"/>
     </row>
     <row r="78" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A78" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B78" s="23" t="s">
-        <v>161</v>
+        <v>93</v>
       </c>
       <c r="C78" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="E78" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F78" s="33">
         <v>-52.3</v>
@@ -3807,19 +3821,19 @@
     </row>
     <row r="79" spans="1:15" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A79" s="24" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="B79" s="23" t="s">
-        <v>162</v>
+        <v>94</v>
       </c>
       <c r="C79" s="22" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="E79" s="32" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="F79" s="33">
         <v>-48.3</v>
@@ -3832,21 +3846,21 @@
       <c r="O79" s="3"/>
     </row>
     <row r="80" spans="1:15" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A80" s="41" t="s">
-        <v>163</v>
-      </c>
-      <c r="B80" s="42"/>
-      <c r="C80" s="43"/>
+      <c r="A80" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="B80" s="46"/>
+      <c r="C80" s="47"/>
       <c r="D80" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="E80" s="48" t="s">
-        <v>174</v>
-      </c>
-      <c r="F80" s="49"/>
-      <c r="G80" s="50"/>
-      <c r="H80" s="51"/>
-      <c r="I80" s="52"/>
+        <v>105</v>
+      </c>
+      <c r="E80" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="F80" s="52"/>
+      <c r="G80" s="43"/>
+      <c r="H80" s="53"/>
+      <c r="I80" s="54"/>
     </row>
     <row r="81" spans="6:6" x14ac:dyDescent="0.4">
       <c r="F81" s="21"/>
@@ -3923,10 +3937,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A287566D-3E57-43AF-AD99-F938555C1D94}">
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="40.59765625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="24.59765625" style="1" customWidth="1"/>
     <col min="2" max="2" width="56.59765625" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.59765625" style="1" customWidth="1"/>
     <col min="4" max="4" width="16.59765625" style="14" customWidth="1"/>
@@ -3934,35 +3948,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="53" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
+      <c r="A1" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
       <c r="E1"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="40"/>
+      <c r="B2" s="55" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="41"/>
     </row>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>3</v>
+        <v>122</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D3" s="17">
         <v>-53.7</v>
@@ -3971,13 +3985,13 @@
     </row>
     <row r="4" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D4" s="17">
         <v>-50.2</v>
@@ -3986,13 +4000,13 @@
     </row>
     <row r="5" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
-        <v>5</v>
+        <v>124</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D5" s="17">
         <v>-46.5</v>
@@ -4001,13 +4015,13 @@
     </row>
     <row r="6" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D6" s="17">
         <v>-45.5</v>
@@ -4016,13 +4030,13 @@
     </row>
     <row r="7" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>126</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D7" s="17">
         <v>-48.4</v>
@@ -4031,13 +4045,13 @@
     </row>
     <row r="8" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D8" s="17">
         <v>-50.1</v>
@@ -4046,13 +4060,13 @@
     </row>
     <row r="9" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
-        <v>9</v>
+        <v>128</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D9" s="17">
         <v>-51.7</v>
@@ -4061,13 +4075,13 @@
     </row>
     <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
-        <v>10</v>
+        <v>129</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D10" s="17">
         <v>-47.8</v>
@@ -4076,13 +4090,13 @@
     </row>
     <row r="11" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D11" s="17">
         <v>-46.1</v>
@@ -4091,13 +4105,13 @@
     </row>
     <row r="12" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
-        <v>12</v>
+        <v>131</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D12" s="17">
         <v>-54.8</v>
@@ -4106,13 +4120,13 @@
     </row>
     <row r="13" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
-        <v>13</v>
+        <v>132</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D13" s="17">
         <v>-49.1</v>
@@ -4121,13 +4135,13 @@
     </row>
     <row r="14" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D14" s="17">
         <v>-49.5</v>
@@ -4136,13 +4150,13 @@
     </row>
     <row r="15" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
-        <v>15</v>
+        <v>134</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D15" s="17">
         <v>-45.7</v>
@@ -4151,13 +4165,13 @@
     </row>
     <row r="16" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D16" s="17">
         <v>-46.1</v>
@@ -4166,13 +4180,13 @@
     </row>
     <row r="17" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
-        <v>17</v>
+        <v>136</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D17" s="17">
         <v>-49.5</v>
@@ -4181,13 +4195,13 @@
     </row>
     <row r="18" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
-        <v>18</v>
+        <v>137</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D18" s="17">
         <v>-51</v>
@@ -4196,13 +4210,13 @@
     </row>
     <row r="19" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
-        <v>19</v>
+        <v>138</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D19" s="17">
         <v>-48.8</v>
@@ -4211,13 +4225,13 @@
     </row>
     <row r="20" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
-        <v>20</v>
+        <v>139</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D20" s="17">
         <v>-53.4</v>
@@ -4226,13 +4240,13 @@
     </row>
     <row r="21" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
-        <v>21</v>
+        <v>140</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D21" s="17">
         <v>-48</v>
@@ -4241,13 +4255,13 @@
     </row>
     <row r="22" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
-        <v>22</v>
+        <v>141</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D22" s="17">
         <v>-53.4</v>
@@ -4256,13 +4270,13 @@
     </row>
     <row r="23" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
-        <v>23</v>
+        <v>142</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D23" s="17">
         <v>-51.3</v>
@@ -4271,13 +4285,13 @@
     </row>
     <row r="24" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
-        <v>24</v>
+        <v>143</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D24" s="17">
         <v>-50.4</v>
@@ -4286,13 +4300,13 @@
     </row>
     <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
-        <v>25</v>
+        <v>144</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D25" s="17">
         <v>-51.2</v>
@@ -4301,13 +4315,13 @@
     </row>
     <row r="26" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
-        <v>26</v>
+        <v>145</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D26" s="17">
         <v>-45.7</v>
@@ -4316,13 +4330,13 @@
     </row>
     <row r="27" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
-        <v>27</v>
+        <v>146</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D27" s="17">
         <v>-49.9</v>
@@ -4331,13 +4345,13 @@
     </row>
     <row r="28" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>28</v>
+        <v>147</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D28" s="17">
         <v>-51.1</v>
@@ -4346,13 +4360,13 @@
     </row>
     <row r="29" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>29</v>
+        <v>148</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D29" s="17">
         <v>-49.1</v>
@@ -4361,13 +4375,13 @@
     </row>
     <row r="30" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
-        <v>30</v>
+        <v>149</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D30" s="16">
         <v>-56.4</v>
@@ -4376,13 +4390,13 @@
     </row>
     <row r="31" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
-        <v>31</v>
+        <v>150</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D31" s="17">
         <v>-48.9</v>
@@ -4391,13 +4405,13 @@
     </row>
     <row r="32" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D32" s="16">
         <v>-43.3</v>
@@ -4406,13 +4420,13 @@
     </row>
     <row r="33" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
-        <v>33</v>
+        <v>152</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D33" s="17">
         <v>-49.6</v>
@@ -4421,13 +4435,13 @@
     </row>
     <row r="34" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
-        <v>34</v>
+        <v>153</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D34" s="17">
         <v>-45</v>
@@ -4436,13 +4450,13 @@
     </row>
     <row r="35" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
-        <v>35</v>
+        <v>154</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D35" s="17">
         <v>-49.1</v>
@@ -4451,13 +4465,13 @@
     </row>
     <row r="36" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
-        <v>36</v>
+        <v>155</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D36" s="17">
         <v>-46.3</v>
@@ -4466,13 +4480,13 @@
     </row>
     <row r="37" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
-        <v>37</v>
+        <v>156</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D37" s="17">
         <v>-50.3</v>
@@ -4481,13 +4495,13 @@
     </row>
     <row r="38" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
-        <v>38</v>
+        <v>157</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D38" s="17">
         <v>-43.9</v>
@@ -4496,13 +4510,13 @@
     </row>
     <row r="39" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
-        <v>39</v>
+        <v>158</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D39" s="17">
         <v>-48.3</v>
@@ -4511,13 +4525,13 @@
     </row>
     <row r="40" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
-        <v>40</v>
+        <v>159</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>74</v>
+        <v>7</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D40" s="17">
         <v>-51.9</v>
@@ -4526,13 +4540,13 @@
     </row>
     <row r="41" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
-        <v>41</v>
+        <v>160</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D41" s="17">
         <v>-52.4</v>
@@ -4541,13 +4555,13 @@
     </row>
     <row r="42" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
-        <v>42</v>
+        <v>161</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D42" s="17">
         <v>-46</v>
@@ -4556,13 +4570,13 @@
     </row>
     <row r="43" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
-        <v>43</v>
+        <v>162</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D43" s="17">
         <v>-48.8</v>
@@ -4571,13 +4585,13 @@
     </row>
     <row r="44" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="4" t="s">
-        <v>44</v>
+        <v>163</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D44" s="17">
         <v>-53.4</v>
@@ -4586,13 +4600,13 @@
     </row>
     <row r="45" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
-        <v>45</v>
+        <v>164</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D45" s="17">
         <v>-44.2</v>
@@ -4601,13 +4615,13 @@
     </row>
     <row r="46" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
-        <v>46</v>
+        <v>165</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D46" s="17">
         <v>-52.4</v>
@@ -4616,13 +4630,13 @@
     </row>
     <row r="47" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="4" t="s">
-        <v>47</v>
+        <v>166</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D47" s="17">
         <v>-46.4</v>
@@ -4631,13 +4645,13 @@
     </row>
     <row r="48" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
-        <v>48</v>
+        <v>167</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D48" s="17">
         <v>-49.4</v>
@@ -4646,13 +4660,13 @@
     </row>
     <row r="49" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="4" t="s">
-        <v>49</v>
+        <v>168</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D49" s="17">
         <v>-50.9</v>
@@ -4661,13 +4675,13 @@
     </row>
     <row r="50" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
-        <v>50</v>
+        <v>169</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D50" s="17">
         <v>-47.9</v>
@@ -4676,13 +4690,13 @@
     </row>
     <row r="51" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="4" t="s">
-        <v>51</v>
+        <v>170</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D51" s="17">
         <v>-49.9</v>
@@ -4691,13 +4705,13 @@
     </row>
     <row r="52" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D52" s="17">
         <v>-46.3</v>
@@ -4706,13 +4720,13 @@
     </row>
     <row r="53" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A53" s="4" t="s">
-        <v>53</v>
+        <v>172</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D53" s="17">
         <v>-50.5</v>
@@ -4721,13 +4735,13 @@
     </row>
     <row r="54" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
-        <v>54</v>
+        <v>173</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D54" s="17">
         <v>-50.2</v>
@@ -4736,13 +4750,13 @@
     </row>
     <row r="55" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>55</v>
+        <v>174</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D55" s="17">
         <v>-50.2</v>
@@ -4751,13 +4765,13 @@
     </row>
     <row r="56" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>56</v>
+        <v>175</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D56" s="17">
         <v>-49.7</v>
@@ -4766,13 +4780,13 @@
     </row>
     <row r="57" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
-        <v>57</v>
+        <v>176</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D57" s="17">
         <v>-49.4</v>
@@ -4781,13 +4795,13 @@
     </row>
     <row r="58" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A58" s="4" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D58" s="17">
         <v>-45</v>
@@ -4796,13 +4810,13 @@
     </row>
     <row r="59" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
-        <v>59</v>
+        <v>178</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D59" s="17">
         <v>-49.4</v>
@@ -4811,13 +4825,13 @@
     </row>
     <row r="60" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D60" s="17">
         <v>-43.9</v>
@@ -4826,13 +4840,13 @@
     </row>
     <row r="61" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>61</v>
+        <v>180</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D61" s="17">
         <v>-50.2</v>
@@ -4841,13 +4855,13 @@
     </row>
     <row r="62" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>62</v>
+        <v>181</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D62" s="17">
         <v>-52.2</v>
@@ -4856,13 +4870,13 @@
     </row>
     <row r="63" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
-        <v>63</v>
+        <v>182</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D63" s="17">
         <v>-47.3</v>
@@ -4870,13 +4884,13 @@
     </row>
     <row r="64" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
-        <v>64</v>
+        <v>183</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D64" s="17">
         <v>-50.2</v>
@@ -4884,13 +4898,13 @@
     </row>
     <row r="65" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A65" s="4" t="s">
-        <v>65</v>
+        <v>184</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D65" s="17">
         <v>-46.5</v>
@@ -4898,13 +4912,13 @@
     </row>
     <row r="66" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A66" s="4" t="s">
-        <v>66</v>
+        <v>185</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D66" s="17">
         <v>-52.5</v>
@@ -4912,13 +4926,13 @@
     </row>
     <row r="67" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A67" s="4" t="s">
-        <v>67</v>
+        <v>186</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D67" s="17">
         <v>-46.6</v>
@@ -4926,29 +4940,43 @@
     </row>
     <row r="68" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A68" s="4" t="s">
-        <v>68</v>
+        <v>187</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="D68" s="17">
         <v>-45.9</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="C69" s="48" t="s">
-        <v>80</v>
-      </c>
-      <c r="D69" s="50"/>
+    <row r="69" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A69" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B69" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D69" s="17">
+        <v>-49.9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A70" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C70" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="43"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D68">
@@ -4957,10 +4985,10 @@
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="C70:D70"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="D3:D68">
+  <conditionalFormatting sqref="D3:D69">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>